<commit_message>
Columna CIS har fået status Godkendt
</commit_message>
<xml_diff>
--- a/html/Sygehus-EPJ-systemer_excel.XLSX
+++ b/html/Sygehus-EPJ-systemer_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0C2710-A437-4F1E-9191-B279DEE96E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D440D04-F03A-4C32-8269-8CBA58923267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Opdateret d. 06-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Sygehus_EPJ_systemer">'Opdateret d. 06-03-2026'!$A$1:$F$107</definedName>
+    <definedName name="Sygehus_EPJ_systemer">'Opdateret d. 06-03-2026'!$A$1:$F$111</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="159">
   <si>
     <t>Standard</t>
   </si>
@@ -263,6 +263,12 @@
     <t>XDIS05 (XD0533L)</t>
   </si>
   <si>
+    <t>BookingConfirmation</t>
+  </si>
+  <si>
+    <t>XDIS13 (XD1333L)</t>
+  </si>
+  <si>
     <t>MunicipalityLetter</t>
   </si>
   <si>
@@ -299,6 +305,12 @@
     <t>XREF01 (XH0131R)</t>
   </si>
   <si>
+    <t>XrayRequest</t>
+  </si>
+  <si>
+    <t>XREF02 (XH0231R)</t>
+  </si>
+  <si>
     <t>LaboratoryReport</t>
   </si>
   <si>
@@ -459,12 +471,6 @@
   </si>
   <si>
     <t>XDIS32 (XD3234L)</t>
-  </si>
-  <si>
-    <t>XrayRequest</t>
-  </si>
-  <si>
-    <t>XREF02 (XH0231R)</t>
   </si>
   <si>
     <t>PrivateSpecialistReferral</t>
@@ -836,7 +842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1450,9 +1456,6 @@
       <c r="D39" t="s">
         <v>9</v>
       </c>
-      <c r="F39" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
@@ -1467,9 +1470,6 @@
       <c r="D40" t="s">
         <v>9</v>
       </c>
-      <c r="E40" t="s">
-        <v>9</v>
-      </c>
       <c r="F40" t="s">
         <v>9</v>
       </c>
@@ -1484,6 +1484,12 @@
       <c r="C41" t="s">
         <v>8</v>
       </c>
+      <c r="D41" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41" t="s">
+        <v>9</v>
+      </c>
       <c r="F41" t="s">
         <v>9</v>
       </c>
@@ -1498,7 +1504,7 @@
       <c r="C42" t="s">
         <v>8</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1512,11 +1518,8 @@
       <c r="C43" t="s">
         <v>8</v>
       </c>
-      <c r="D43" t="s">
-        <v>9</v>
-      </c>
-      <c r="F43" t="s">
-        <v>14</v>
+      <c r="E43" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1532,6 +1535,9 @@
       <c r="D44" t="s">
         <v>9</v>
       </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -1543,30 +1549,30 @@
       <c r="C45" t="s">
         <v>8</v>
       </c>
-      <c r="F45" t="s">
+      <c r="D45" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C46" t="s">
         <v>8</v>
       </c>
-      <c r="F46" t="s">
+      <c r="D46" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C47" t="s">
         <v>8</v>
@@ -1577,10 +1583,10 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C48" t="s">
         <v>8</v>
@@ -1591,10 +1597,10 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C49" t="s">
         <v>8</v>
@@ -1605,10 +1611,10 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C50" t="s">
         <v>8</v>
@@ -1619,10 +1625,10 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B51" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C51" t="s">
         <v>8</v>
@@ -1633,10 +1639,10 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C52" t="s">
         <v>8</v>
@@ -1647,16 +1653,16 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>6</v>
+        <v>104</v>
       </c>
       <c r="B53" t="s">
-        <v>7</v>
+        <v>105</v>
       </c>
       <c r="C53" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="F53" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -1664,10 +1670,10 @@
         <v>104</v>
       </c>
       <c r="B54" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C54" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="F54" t="s">
         <v>9</v>
@@ -1675,49 +1681,43 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B55" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C55" t="s">
-        <v>103</v>
-      </c>
-      <c r="D55" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F55" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
+        <v>109</v>
       </c>
       <c r="C56" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F56" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C57" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D57" t="s">
-        <v>9</v>
-      </c>
-      <c r="E57" t="s">
         <v>9</v>
       </c>
       <c r="F57" t="s">
@@ -1726,49 +1726,52 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C58" t="s">
-        <v>103</v>
-      </c>
-      <c r="D58" t="s">
-        <v>9</v>
-      </c>
-      <c r="E58" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F58" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>106</v>
+        <v>17</v>
       </c>
       <c r="B59" t="s">
-        <v>107</v>
+        <v>18</v>
       </c>
       <c r="C59" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D59" t="s">
+        <v>9</v>
+      </c>
+      <c r="E59" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B60" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C60" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D60" t="s">
+        <v>9</v>
+      </c>
+      <c r="E60" t="s">
         <v>9</v>
       </c>
       <c r="F60" t="s">
@@ -1777,27 +1780,27 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
       <c r="B61" t="s">
-        <v>23</v>
+        <v>111</v>
       </c>
       <c r="C61" t="s">
-        <v>103</v>
-      </c>
-      <c r="E61" t="s">
-        <v>24</v>
+        <v>107</v>
+      </c>
+      <c r="D61" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B62" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C62" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D62" t="s">
         <v>9</v>
@@ -1808,13 +1811,13 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B63" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C63" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E63" t="s">
         <v>24</v>
@@ -1822,13 +1825,13 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B64" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C64" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D64" t="s">
         <v>9</v>
@@ -1839,27 +1842,30 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B65" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C65" t="s">
-        <v>103</v>
-      </c>
-      <c r="F65" t="s">
-        <v>9</v>
+        <v>107</v>
+      </c>
+      <c r="E65" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B66" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C66" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D66" t="s">
+        <v>9</v>
       </c>
       <c r="F66" t="s">
         <v>9</v>
@@ -1867,13 +1873,13 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B67" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C67" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F67" t="s">
         <v>9</v>
@@ -1881,16 +1887,13 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>109</v>
+        <v>37</v>
       </c>
       <c r="C68" t="s">
-        <v>103</v>
-      </c>
-      <c r="D68" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F68" t="s">
         <v>9</v>
@@ -1898,19 +1901,13 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="B69" t="s">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>103</v>
-      </c>
-      <c r="D69" t="s">
-        <v>9</v>
-      </c>
-      <c r="E69" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F69" t="s">
         <v>9</v>
@@ -1918,18 +1915,15 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>42</v>
+        <v>112</v>
       </c>
       <c r="B70" t="s">
-        <v>43</v>
+        <v>113</v>
       </c>
       <c r="C70" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D70" t="s">
-        <v>9</v>
-      </c>
-      <c r="E70" t="s">
         <v>9</v>
       </c>
       <c r="F70" t="s">
@@ -1938,13 +1932,13 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>44</v>
+        <v>114</v>
       </c>
       <c r="B71" t="s">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="C71" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D71" t="s">
         <v>9</v>
@@ -1958,15 +1952,18 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="B72" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="C72" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D72" t="s">
+        <v>9</v>
+      </c>
+      <c r="E72" t="s">
         <v>9</v>
       </c>
       <c r="F72" t="s">
@@ -1975,13 +1972,19 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>114</v>
+        <v>44</v>
       </c>
       <c r="B73" t="s">
-        <v>115</v>
+        <v>45</v>
       </c>
       <c r="C73" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D73" t="s">
+        <v>9</v>
+      </c>
+      <c r="E73" t="s">
+        <v>9</v>
       </c>
       <c r="F73" t="s">
         <v>9</v>
@@ -1995,7 +1998,7 @@
         <v>117</v>
       </c>
       <c r="C74" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D74" t="s">
         <v>9</v>
@@ -2012,10 +2015,7 @@
         <v>119</v>
       </c>
       <c r="C75" t="s">
-        <v>103</v>
-      </c>
-      <c r="D75" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F75" t="s">
         <v>9</v>
@@ -2023,13 +2023,16 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="B76" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C76" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D76" t="s">
+        <v>9</v>
       </c>
       <c r="F76" t="s">
         <v>9</v>
@@ -2037,13 +2040,13 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="B77" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
       <c r="C77" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D77" t="s">
         <v>9</v>
@@ -2054,19 +2057,13 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B78" t="s">
-        <v>57</v>
+        <v>124</v>
       </c>
       <c r="C78" t="s">
-        <v>103</v>
-      </c>
-      <c r="D78" t="s">
-        <v>24</v>
-      </c>
-      <c r="E78" t="s">
-        <v>24</v>
+        <v>107</v>
       </c>
       <c r="F78" t="s">
         <v>9</v>
@@ -2074,13 +2071,16 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B79" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C79" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D79" t="s">
+        <v>9</v>
       </c>
       <c r="F79" t="s">
         <v>9</v>
@@ -2088,16 +2088,19 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B80" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C80" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D80" t="s">
+        <v>24</v>
       </c>
       <c r="E80" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F80" t="s">
         <v>9</v>
@@ -2105,16 +2108,13 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="B81" t="s">
-        <v>122</v>
+        <v>59</v>
       </c>
       <c r="C81" t="s">
-        <v>103</v>
-      </c>
-      <c r="D81" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F81" t="s">
         <v>9</v>
@@ -2122,13 +2122,16 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="B82" t="s">
-        <v>124</v>
+        <v>60</v>
       </c>
       <c r="C82" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
       </c>
       <c r="F82" t="s">
         <v>9</v>
@@ -2142,7 +2145,10 @@
         <v>126</v>
       </c>
       <c r="C83" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D83" t="s">
+        <v>9</v>
       </c>
       <c r="F83" t="s">
         <v>9</v>
@@ -2156,7 +2162,7 @@
         <v>128</v>
       </c>
       <c r="C84" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F84" t="s">
         <v>9</v>
@@ -2170,7 +2176,7 @@
         <v>130</v>
       </c>
       <c r="C85" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F85" t="s">
         <v>9</v>
@@ -2184,10 +2190,7 @@
         <v>132</v>
       </c>
       <c r="C86" t="s">
-        <v>103</v>
-      </c>
-      <c r="D86" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F86" t="s">
         <v>9</v>
@@ -2195,19 +2198,13 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="B87" t="s">
-        <v>62</v>
+        <v>134</v>
       </c>
       <c r="C87" t="s">
-        <v>103</v>
-      </c>
-      <c r="D87" t="s">
-        <v>9</v>
-      </c>
-      <c r="E87" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="F87" t="s">
         <v>9</v>
@@ -2215,13 +2212,16 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>63</v>
+        <v>135</v>
       </c>
       <c r="B88" t="s">
-        <v>64</v>
+        <v>136</v>
       </c>
       <c r="C88" t="s">
-        <v>103</v>
+        <v>107</v>
+      </c>
+      <c r="D88" t="s">
+        <v>9</v>
       </c>
       <c r="F88" t="s">
         <v>9</v>
@@ -2229,81 +2229,78 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B89" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C89" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D89" t="s">
+        <v>9</v>
+      </c>
+      <c r="E89" t="s">
+        <v>9</v>
+      </c>
+      <c r="F89" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B90" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C90" t="s">
-        <v>103</v>
-      </c>
-      <c r="D90" t="s">
+        <v>107</v>
+      </c>
+      <c r="F90" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B91" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C91" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D91" t="s">
-        <v>9</v>
-      </c>
-      <c r="F91" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B92" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C92" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D92" t="s">
-        <v>9</v>
-      </c>
-      <c r="F92" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B93" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C93" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D93" t="s">
         <v>9</v>
-      </c>
-      <c r="E93" t="s">
-        <v>14</v>
       </c>
       <c r="F93" t="s">
         <v>9</v>
@@ -2311,33 +2308,36 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="B94" t="s">
-        <v>134</v>
+        <v>74</v>
       </c>
       <c r="C94" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D94" t="s">
+        <v>9</v>
+      </c>
+      <c r="F94" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>135</v>
+        <v>75</v>
       </c>
       <c r="B95" t="s">
-        <v>136</v>
+        <v>76</v>
       </c>
       <c r="C95" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D95" t="s">
         <v>9</v>
       </c>
       <c r="E95" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F95" t="s">
         <v>9</v>
@@ -2345,30 +2345,27 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>137</v>
+        <v>77</v>
       </c>
       <c r="B96" t="s">
-        <v>138</v>
+        <v>78</v>
       </c>
       <c r="C96" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D96" t="s">
-        <v>9</v>
-      </c>
-      <c r="F96" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>139</v>
+        <v>79</v>
       </c>
       <c r="B97" t="s">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="C97" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D97" t="s">
         <v>9</v>
@@ -2376,35 +2373,32 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B98" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C98" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D98" t="s">
-        <v>9</v>
-      </c>
-      <c r="E98" t="s">
-        <v>9</v>
-      </c>
-      <c r="F98" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B99" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C99" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D99" t="s">
+        <v>9</v>
+      </c>
+      <c r="E99" t="s">
         <v>9</v>
       </c>
       <c r="F99" t="s">
@@ -2413,13 +2407,13 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="B100" t="s">
-        <v>88</v>
+        <v>142</v>
       </c>
       <c r="C100" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D100" t="s">
         <v>9</v>
@@ -2430,13 +2424,13 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>89</v>
+        <v>143</v>
       </c>
       <c r="B101" t="s">
-        <v>90</v>
+        <v>144</v>
       </c>
       <c r="C101" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D101" t="s">
         <v>9</v>
@@ -2450,9 +2444,15 @@
         <v>146</v>
       </c>
       <c r="C102" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D102" t="s">
+        <v>9</v>
+      </c>
+      <c r="E102" t="s">
+        <v>9</v>
+      </c>
+      <c r="F102" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2464,21 +2464,24 @@
         <v>148</v>
       </c>
       <c r="C103" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D103" t="s">
+        <v>9</v>
+      </c>
+      <c r="F103" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>149</v>
+        <v>89</v>
       </c>
       <c r="B104" t="s">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="C104" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D104" t="s">
         <v>9</v>
@@ -2489,43 +2492,102 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>151</v>
+        <v>91</v>
       </c>
       <c r="B105" t="s">
-        <v>152</v>
+        <v>92</v>
       </c>
       <c r="C105" t="s">
-        <v>103</v>
-      </c>
-      <c r="F105" t="s">
+        <v>107</v>
+      </c>
+      <c r="D105" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>153</v>
+        <v>93</v>
       </c>
       <c r="B106" t="s">
-        <v>154</v>
+        <v>94</v>
       </c>
       <c r="C106" t="s">
-        <v>103</v>
-      </c>
-      <c r="F106" t="s">
+        <v>107</v>
+      </c>
+      <c r="D106" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
+        <v>149</v>
+      </c>
+      <c r="B107" t="s">
+        <v>150</v>
+      </c>
+      <c r="C107" t="s">
+        <v>107</v>
+      </c>
+      <c r="D107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>151</v>
+      </c>
+      <c r="B108" t="s">
+        <v>152</v>
+      </c>
+      <c r="C108" t="s">
+        <v>107</v>
+      </c>
+      <c r="D108" t="s">
+        <v>9</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>153</v>
+      </c>
+      <c r="B109" t="s">
+        <v>154</v>
+      </c>
+      <c r="C109" t="s">
+        <v>107</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
         <v>155</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B110" t="s">
         <v>156</v>
       </c>
-      <c r="C107" t="s">
-        <v>103</v>
-      </c>
-      <c r="F107" t="s">
+      <c r="C110" t="s">
+        <v>107</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>157</v>
+      </c>
+      <c r="B111" t="s">
+        <v>158</v>
+      </c>
+      <c r="C111" t="s">
+        <v>107</v>
+      </c>
+      <c r="F111" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>